<commit_message>
Sinh file thuc hanh tung bai Hoc hom nay
</commit_message>
<xml_diff>
--- a/downloads/daily/b01-freeze.xlsx
+++ b/downloads/daily/b01-freeze.xlsx
@@ -512,7 +512,7 @@
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>1. Chọn ô A2 (ngay dưới hàng tiêu đề).</t>
+          <t>1. Chọn ô A5 (ngay dưới hàng tiêu đề ở dòng 4).</t>
         </is>
       </c>
     </row>
@@ -526,7 +526,7 @@
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>3. Cuộn xuống: hàng 1 đứng yên.</t>
+          <t>3. Cuộn xuống: hàng 4 đứng yên.</t>
         </is>
       </c>
     </row>

</xml_diff>